<commit_message>
Educacion en la vista Nacional con el formato regional (Matricula de 0 a 24, Rezago escolar por sexo y por edad) y Rezago de 6 a 21 por sexo; informes reconstruidos
</commit_message>
<xml_diff>
--- a/output/graficos_nacionales/plot_nacional_serie_e_mat_a_2018.xlsx
+++ b/output/graficos_nacionales/plot_nacional_serie_e_mat_a_2018.xlsx
@@ -6,58 +6,154 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Serie" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Metadata" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tramos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Serie" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Regiones" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Serie'!$A$1:$B$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Regiones'!$A$1:$C$17</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+  <si>
+    <t xml:space="preserve">Grupo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chile (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mujeres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hombres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha de creación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-01 15:12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIT - MDSF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imagen asociada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">plot_nacional_serie_e_mat_a_2018.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E_MAT_a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unidad territorial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chile (Nacional)</t>
+  </si>
   <si>
     <t xml:space="preserve">Año</t>
   </si>
   <si>
-    <t xml:space="preserve">Valor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fecha de creación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-18 11:58</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIT - MDSF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Imagen asociada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">plot_nacional_serie_e_mat_a_2018.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indicador</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tasa de matrícula de 0 a 24 años</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unidad territorial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chile (Nacional)</t>
-  </si>
-  <si>
     <t xml:space="preserve">2018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tramo de edad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 a 1 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 a 3 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 a 5 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 a 13 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 a 17 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18 a 24 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Región</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matrícula (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diferencia con el país (pts)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarapacá</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Antofagasta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atacama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coquimbo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valparaíso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metropolitana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O’Higgins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ñuble</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biobío</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Araucanía</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Los Ríos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Los Lagos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aysén</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Magallanes</t>
   </si>
 </sst>
 </file>
@@ -423,7 +519,7 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="10.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -435,63 +531,31 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>2018</v>
+      <c r="A2" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>71.58</v>
+        <v>71.6</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2019</v>
+      <c r="A3" s="2" t="s">
+        <v>3</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>72.52</v>
+        <v>72.3</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>2020</v>
+      <c r="A4" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>74.1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>72.98</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>74.43</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>71.32</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>76.09</v>
+        <v>70.9</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B8"/>
+  <autoFilter ref="A1:B4"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
@@ -508,62 +572,418 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="15.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="11.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>51.9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>92.3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>97.6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>94.7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>47.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B7"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="11.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>71.6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>72.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>74.1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>74.4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>71.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>76.1</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B8"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="15.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="15.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="30.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>70.9</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>-0.7</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>68.6</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>74.7</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>73.4</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>70.3</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>-1.3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>73.1</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>73.8</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>74.3</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>4.4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>73.8</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>74.9</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>74.3</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>77.4</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>3.4</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C17"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>